<commit_message>
Phase 4: H-032 printed-precision stale rule, verifier re-frozen (verifier-v1); facts check on dev filings
Freeze reopened once with the owner's approval (D-061): a named filing's other value given at the
answer's printed precision is stale_value; 0.5% tolerance unchanged elsewhere. BAC unit test; full
dev re-run (only FG-0205 T2 changed); new freeze manifest and pinned hash. Facts check on dev
filings, report only.
</commit_message>
<xml_diff>
--- a/review/verifier_dev_verifier_v2.xlsx
+++ b/review/verifier_dev_verifier_v2.xlsx
@@ -7174,13 +7174,17 @@
       </c>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>pass</t>
-        </is>
-      </c>
-      <c r="L97" s="2" t="inlineStr"/>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>stale_value [xbrl]: 2.967e+12 is another filing's value for 2024</t>
+        </is>
+      </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>missed seeded error</t>
+          <t>block</t>
         </is>
       </c>
       <c r="N97" s="2" t="inlineStr"/>
@@ -17809,13 +17813,17 @@
       </c>
       <c r="K250" s="2" t="inlineStr">
         <is>
-          <t>pass</t>
-        </is>
-      </c>
-      <c r="L250" s="2" t="inlineStr"/>
+          <t>block</t>
+        </is>
+      </c>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>stale_value [xbrl]: 2.967e+12 is another filing's value for 2024</t>
+        </is>
+      </c>
       <c r="M250" s="2" t="inlineStr">
         <is>
-          <t>missed seeded error</t>
+          <t>block</t>
         </is>
       </c>
       <c r="N250" s="2" t="inlineStr"/>

</xml_diff>